<commit_message>
#41 Client BOM update.
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.4/BOM/Client -BOM IoT-Button-v1.4.xlsx
+++ b/Design Files/IoT-Button-v1.4/BOM/Client -BOM IoT-Button-v1.4.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20413"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Button-v1.4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912B4A5B-94F6-4417-B01D-1ACDADFA1686}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="156">
   <si>
     <t>#</t>
   </si>
@@ -493,7 +492,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -799,7 +798,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -836,103 +835,100 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1221,22 +1217,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.85546875" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.42578125" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1248,10 +1244,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1282,7 +1278,7 @@
       <c r="J2" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="21" t="s">
         <v>133</v>
       </c>
       <c r="L2" s="5" t="s">
@@ -1316,11 +1312,13 @@
       <c r="I3" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="J3" s="7"/>
-      <c r="K3" s="23">
+      <c r="J3" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="K3" s="22">
         <v>5</v>
       </c>
-      <c r="L3" s="45"/>
+      <c r="L3" s="37"/>
     </row>
     <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -1331,29 +1329,31 @@
       <c r="C4" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="J4" s="15"/>
-      <c r="K4" s="24">
-        <v>1</v>
-      </c>
-      <c r="L4" s="19" t="s">
+      <c r="J4" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K4" s="23">
+        <v>1</v>
+      </c>
+      <c r="L4" s="18" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1366,29 +1366,31 @@
       <c r="C5" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="H5" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="I5" s="18" t="s">
+      <c r="I5" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="J5" s="17"/>
-      <c r="K5" s="25">
-        <v>1</v>
-      </c>
-      <c r="L5" s="19" t="s">
+      <c r="J5" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K5" s="24">
+        <v>1</v>
+      </c>
+      <c r="L5" s="18" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1419,11 +1421,13 @@
       <c r="I6" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="J6" s="9"/>
-      <c r="K6" s="26">
+      <c r="J6" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K6" s="25">
         <v>14</v>
       </c>
-      <c r="L6" s="19"/>
+      <c r="L6" s="18"/>
     </row>
     <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -1452,11 +1456,13 @@
       <c r="I7" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="J7" s="7"/>
-      <c r="K7" s="23">
-        <v>1</v>
-      </c>
-      <c r="L7" s="45"/>
+      <c r="J7" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K7" s="22">
+        <v>1</v>
+      </c>
+      <c r="L7" s="37"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1467,29 +1473,31 @@
       <c r="C8" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="J8" s="9"/>
-      <c r="K8" s="26">
-        <v>1</v>
-      </c>
-      <c r="L8" s="19" t="s">
+      <c r="J8" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K8" s="23">
+        <v>1</v>
+      </c>
+      <c r="L8" s="18" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1520,11 +1528,13 @@
       <c r="I9" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="J9" s="7"/>
-      <c r="K9" s="23">
-        <v>1</v>
-      </c>
-      <c r="L9" s="45"/>
+      <c r="J9" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K9" s="22">
+        <v>1</v>
+      </c>
+      <c r="L9" s="37"/>
     </row>
     <row r="10" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
@@ -1553,11 +1563,13 @@
       <c r="I10" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="J10" s="7"/>
-      <c r="K10" s="26">
-        <v>1</v>
-      </c>
-      <c r="L10" s="19"/>
+      <c r="J10" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K10" s="25">
+        <v>1</v>
+      </c>
+      <c r="L10" s="18"/>
     </row>
     <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
@@ -1586,11 +1598,13 @@
       <c r="I11" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="J11" s="7"/>
-      <c r="K11" s="23">
-        <v>1</v>
-      </c>
-      <c r="L11" s="45"/>
+      <c r="J11" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K11" s="22">
+        <v>1</v>
+      </c>
+      <c r="L11" s="37"/>
     </row>
     <row r="12" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -1619,11 +1633,13 @@
       <c r="I12" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="J12" s="7"/>
-      <c r="K12" s="26">
-        <v>1</v>
-      </c>
-      <c r="L12" s="19"/>
+      <c r="J12" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K12" s="25">
+        <v>1</v>
+      </c>
+      <c r="L12" s="18"/>
     </row>
     <row r="13" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
@@ -1634,29 +1650,31 @@
       <c r="C13" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="G13" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="H13" s="17" t="s">
+      <c r="H13" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="I13" s="18" t="s">
+      <c r="I13" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="J13" s="17"/>
-      <c r="K13" s="25">
-        <v>1</v>
-      </c>
-      <c r="L13" s="45" t="s">
+      <c r="J13" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K13" s="24">
+        <v>1</v>
+      </c>
+      <c r="L13" s="37" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1687,11 +1705,13 @@
       <c r="I14" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="J14" s="9"/>
-      <c r="K14" s="26">
-        <v>1</v>
-      </c>
-      <c r="L14" s="19"/>
+      <c r="J14" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K14" s="25">
+        <v>1</v>
+      </c>
+      <c r="L14" s="18"/>
     </row>
     <row r="15" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
@@ -1702,29 +1722,31 @@
       <c r="C15" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="G15" s="18" t="s">
+      <c r="G15" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="H15" s="17" t="s">
+      <c r="H15" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="I15" s="18" t="s">
+      <c r="I15" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="J15" s="17"/>
-      <c r="K15" s="25">
-        <v>1</v>
-      </c>
-      <c r="L15" s="44" t="s">
+      <c r="J15" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K15" s="24">
+        <v>1</v>
+      </c>
+      <c r="L15" s="36" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1755,11 +1777,13 @@
       <c r="I16" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="J16" s="9"/>
-      <c r="K16" s="26">
+      <c r="J16" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K16" s="25">
         <v>6</v>
       </c>
-      <c r="L16" s="19"/>
+      <c r="L16" s="18"/>
     </row>
     <row r="17" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
@@ -1788,11 +1812,13 @@
       <c r="I17" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="J17" s="7"/>
-      <c r="K17" s="23">
-        <v>1</v>
-      </c>
-      <c r="L17" s="45"/>
+      <c r="J17" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K17" s="22">
+        <v>1</v>
+      </c>
+      <c r="L17" s="37"/>
     </row>
     <row r="18" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
@@ -1803,29 +1829,31 @@
       <c r="C18" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E18" s="16" t="s">
+      <c r="E18" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="15" t="s">
+      <c r="F18" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="G18" s="16" t="s">
+      <c r="G18" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="H18" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="I18" s="16" t="s">
+      <c r="I18" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="J18" s="15"/>
-      <c r="K18" s="24">
-        <v>1</v>
-      </c>
-      <c r="L18" s="19" t="s">
+      <c r="J18" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K18" s="23">
+        <v>1</v>
+      </c>
+      <c r="L18" s="18" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1838,29 +1866,31 @@
       <c r="C19" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="G19" s="18" t="s">
+      <c r="G19" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="H19" s="17" t="s">
+      <c r="H19" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="I19" s="18" t="s">
+      <c r="I19" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="J19" s="17"/>
-      <c r="K19" s="25">
-        <v>1</v>
-      </c>
-      <c r="L19" s="45" t="s">
+      <c r="J19" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K19" s="24">
+        <v>1</v>
+      </c>
+      <c r="L19" s="37" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1873,29 +1903,31 @@
       <c r="C20" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="E20" s="16" t="s">
+      <c r="E20" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="F20" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="G20" s="16" t="s">
+      <c r="G20" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="H20" s="15" t="s">
+      <c r="H20" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="I20" s="16" t="s">
+      <c r="I20" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="J20" s="15"/>
-      <c r="K20" s="24">
-        <v>1</v>
-      </c>
-      <c r="L20" s="19" t="s">
+      <c r="J20" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K20" s="23">
+        <v>1</v>
+      </c>
+      <c r="L20" s="18" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1926,11 +1958,13 @@
       <c r="I21" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="J21" s="7"/>
-      <c r="K21" s="23">
+      <c r="J21" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K21" s="22">
         <v>6</v>
       </c>
-      <c r="L21" s="45"/>
+      <c r="L21" s="37"/>
     </row>
     <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
@@ -1941,29 +1975,31 @@
       <c r="C22" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E22" s="16" t="s">
+      <c r="E22" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="F22" s="15" t="s">
+      <c r="F22" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="G22" s="16" t="s">
+      <c r="G22" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="H22" s="15" t="s">
+      <c r="H22" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="I22" s="16" t="s">
+      <c r="I22" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="J22" s="15"/>
-      <c r="K22" s="24">
+      <c r="J22" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K22" s="23">
         <v>2</v>
       </c>
-      <c r="L22" s="19" t="s">
+      <c r="L22" s="18" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1974,29 +2010,31 @@
         <v>21</v>
       </c>
       <c r="C23" s="12"/>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="E23" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="G23" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="H23" s="17" t="s">
+      <c r="H23" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="I23" s="18" t="s">
+      <c r="I23" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="J23" s="17"/>
-      <c r="K23" s="25">
-        <v>1</v>
-      </c>
-      <c r="L23" s="45" t="s">
+      <c r="J23" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K23" s="24">
+        <v>1</v>
+      </c>
+      <c r="L23" s="37" t="s">
         <v>155</v>
       </c>
     </row>
@@ -2027,11 +2065,13 @@
       <c r="I24" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="J24" s="9"/>
-      <c r="K24" s="26">
-        <v>1</v>
-      </c>
-      <c r="L24" s="19"/>
+      <c r="J24" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K24" s="25">
+        <v>1</v>
+      </c>
+      <c r="L24" s="18"/>
     </row>
     <row r="25" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
@@ -2060,11 +2100,13 @@
       <c r="I25" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="J25" s="7"/>
-      <c r="K25" s="23">
+      <c r="J25" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K25" s="22">
         <v>2</v>
       </c>
-      <c r="L25" s="45"/>
+      <c r="L25" s="37"/>
     </row>
     <row r="26" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
@@ -2093,11 +2135,13 @@
       <c r="I26" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="J26" s="7"/>
-      <c r="K26" s="26">
-        <v>1</v>
-      </c>
-      <c r="L26" s="19"/>
+      <c r="J26" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K26" s="25">
+        <v>1</v>
+      </c>
+      <c r="L26" s="18"/>
     </row>
     <row r="27" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
@@ -2126,11 +2170,13 @@
       <c r="I27" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="J27" s="7"/>
-      <c r="K27" s="23">
-        <v>1</v>
-      </c>
-      <c r="L27" s="45"/>
+      <c r="J27" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K27" s="22">
+        <v>1</v>
+      </c>
+      <c r="L27" s="37"/>
     </row>
     <row r="28" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
@@ -2141,29 +2187,31 @@
       <c r="C28" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E28" s="16" t="s">
+      <c r="E28" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="F28" s="15" t="s">
+      <c r="F28" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="G28" s="16" t="s">
+      <c r="G28" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="H28" s="15" t="s">
+      <c r="H28" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="I28" s="16" t="s">
+      <c r="I28" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="J28" s="15"/>
-      <c r="K28" s="24">
-        <v>1</v>
-      </c>
-      <c r="L28" s="19" t="s">
+      <c r="J28" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K28" s="23">
+        <v>1</v>
+      </c>
+      <c r="L28" s="18" t="s">
         <v>155</v>
       </c>
     </row>
@@ -2194,11 +2242,13 @@
       <c r="I29" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="J29" s="7"/>
-      <c r="K29" s="23">
-        <v>1</v>
-      </c>
-      <c r="L29" s="45"/>
+      <c r="J29" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K29" s="22">
+        <v>1</v>
+      </c>
+      <c r="L29" s="37"/>
     </row>
     <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
@@ -2227,11 +2277,13 @@
       <c r="I30" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="J30" s="29"/>
-      <c r="K30" s="26">
-        <v>1</v>
-      </c>
-      <c r="L30" s="19"/>
+      <c r="J30" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K30" s="25">
+        <v>1</v>
+      </c>
+      <c r="L30" s="18"/>
     </row>
     <row r="31" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="11">
@@ -2256,16 +2308,16 @@
       <c r="H31" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="I31" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="J31" s="30" t="s">
+      <c r="I31" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="J31" s="28" t="s">
         <v>141</v>
       </c>
       <c r="K31" s="7">
         <v>1</v>
       </c>
-      <c r="L31" s="45"/>
+      <c r="L31" s="37"/>
     </row>
     <row r="32" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="11">
@@ -2290,16 +2342,16 @@
       <c r="H32" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="I32" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="J32" s="20" t="s">
+      <c r="I32" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="J32" s="19" t="s">
         <v>141</v>
       </c>
       <c r="K32" s="7">
         <v>1</v>
       </c>
-      <c r="L32" s="45"/>
+      <c r="L32" s="37"/>
     </row>
     <row r="33" spans="2:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="11">
@@ -2327,107 +2379,107 @@
       <c r="I33" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="J33" s="31" t="s">
+      <c r="J33" s="29" t="s">
         <v>146</v>
       </c>
       <c r="K33" s="9">
         <v>1</v>
       </c>
-      <c r="L33" s="19"/>
+      <c r="L33" s="18"/>
     </row>
     <row r="34" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="11">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C34" s="34" t="s">
+      <c r="C34" s="40" t="s">
         <v>147</v>
       </c>
-      <c r="D34" s="35" t="s">
+      <c r="D34" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="E34" s="36" t="s">
+      <c r="E34" s="32" t="s">
         <v>148</v>
       </c>
-      <c r="F34" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="G34" s="37" t="s">
+      <c r="F34" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="G34" s="33" t="s">
         <v>149</v>
       </c>
-      <c r="H34" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="I34" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="J34" s="31" t="s">
+      <c r="H34" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="I34" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="J34" s="29" t="s">
         <v>141</v>
       </c>
       <c r="K34" s="7">
         <v>3</v>
       </c>
-      <c r="L34" s="45"/>
+      <c r="L34" s="37"/>
     </row>
     <row r="35" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="11">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C35" s="38"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="36" t="s">
+      <c r="C35" s="41"/>
+      <c r="D35" s="44"/>
+      <c r="E35" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="F35" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="G35" s="37" t="s">
+      <c r="F35" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="G35" s="33" t="s">
         <v>151</v>
       </c>
-      <c r="H35" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="I35" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="J35" s="32" t="s">
+      <c r="H35" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="I35" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="J35" s="30" t="s">
         <v>141</v>
       </c>
       <c r="K35" s="7">
         <v>2</v>
       </c>
-      <c r="L35" s="45"/>
+      <c r="L35" s="37"/>
     </row>
     <row r="36" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="11">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C36" s="40"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="42" t="s">
+      <c r="C36" s="42"/>
+      <c r="D36" s="45"/>
+      <c r="E36" s="34" t="s">
         <v>152</v>
       </c>
-      <c r="F36" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="G36" s="43" t="s">
+      <c r="F36" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="G36" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="H36" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="I36" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="J36" s="33" t="s">
+      <c r="H36" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="I36" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="J36" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="K36" s="28">
+      <c r="K36" s="27">
         <v>4</v>
       </c>
-      <c r="L36" s="46"/>
+      <c r="L36" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2436,12 +2488,12 @@
     <mergeCell ref="D34:D36"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="J31" r:id="rId1" xr:uid="{B7EC1811-5C7F-4D69-A252-67DD4257F611}"/>
-    <hyperlink ref="J32" r:id="rId2" xr:uid="{232BE579-4A2A-47D7-9240-611BD168F29A}"/>
-    <hyperlink ref="J33" r:id="rId3" xr:uid="{9A10DEDA-5839-4A97-AEFA-9B898C975E56}"/>
-    <hyperlink ref="J34" r:id="rId4" xr:uid="{91E2DC22-8B6A-44DB-A250-4AB4E288516E}"/>
-    <hyperlink ref="J36" r:id="rId5" xr:uid="{136608BC-7283-4E58-97CD-D4144285D524}"/>
-    <hyperlink ref="J35" r:id="rId6" xr:uid="{3D00C71B-8624-4516-B2EF-1745F8146747}"/>
+    <hyperlink ref="J35" r:id="rId1"/>
+    <hyperlink ref="J36" r:id="rId2"/>
+    <hyperlink ref="J34" r:id="rId3"/>
+    <hyperlink ref="J33" r:id="rId4"/>
+    <hyperlink ref="J32" r:id="rId5"/>
+    <hyperlink ref="J31" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>

</xml_diff>

<commit_message>
#41 Fresh Deliverables Generated: Client BOM updated with DNP's.
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.4/BOM/Client -BOM IoT-Button-v1.4.xlsx
+++ b/Design Files/IoT-Button-v1.4/BOM/Client -BOM IoT-Button-v1.4.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Button-v1.4\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\smartmasjid-hardware\Design Files\IoT-Button-v1.4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="161">
   <si>
     <t>#</t>
   </si>
@@ -120,9 +120,6 @@
     <t>Q2</t>
   </si>
   <si>
-    <t>R1</t>
-  </si>
-  <si>
     <t>R3</t>
   </si>
   <si>
@@ -261,9 +258,6 @@
     <t>WS2812B-XF02/W</t>
   </si>
   <si>
-    <t>Sot-23</t>
-  </si>
-  <si>
     <t>SOT-23</t>
   </si>
   <si>
@@ -423,9 +417,6 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>value</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -487,6 +478,30 @@
   </si>
   <si>
     <t>DO NOT POPULATE</t>
+  </si>
+  <si>
+    <t>LED1</t>
+  </si>
+  <si>
+    <t>Emerald 0603 Light Emitting Diodes (LED) ROHS</t>
+  </si>
+  <si>
+    <t>NCD0603G2</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>R1, R8</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>RES SMD 220 OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>RC0603FR-07220RL</t>
   </si>
 </sst>
 </file>
@@ -1219,7 +1234,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1261,28 +1276,28 @@
         <v>16</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>134</v>
+        <v>156</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="K2" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>133</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1298,22 +1313,22 @@
         <v>17</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K3" s="22">
         <v>5</v>
@@ -1323,7 +1338,7 @@
     <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B36" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B38" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -1333,28 +1348,28 @@
         <v>18</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K4" s="23">
         <v>1</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1370,28 +1385,28 @@
         <v>19</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I5" s="17" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K5" s="24">
         <v>1</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1407,22 +1422,22 @@
         <v>20</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K6" s="25">
         <v>14</v>
@@ -1442,22 +1457,22 @@
         <v>21</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K7" s="22">
         <v>1</v>
@@ -1477,28 +1492,28 @@
         <v>22</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K8" s="23">
         <v>1</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1514,22 +1529,22 @@
         <v>23</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K9" s="22">
         <v>1</v>
@@ -1549,22 +1564,22 @@
         <v>24</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K10" s="25">
         <v>1</v>
@@ -1584,22 +1599,22 @@
         <v>25</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J11" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K11" s="22">
         <v>1</v>
@@ -1619,22 +1634,22 @@
         <v>26</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K12" s="25">
         <v>1</v>
@@ -1654,28 +1669,28 @@
         <v>27</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I13" s="17" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J13" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K13" s="24">
         <v>1</v>
       </c>
       <c r="L13" s="37" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1691,22 +1706,22 @@
         <v>28</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J14" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K14" s="25">
         <v>1</v>
@@ -1716,255 +1731,252 @@
     <row r="15" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
-        <f>ROW(B15) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>29</v>
+        <v>153</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>55</v>
+        <v>154</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>98</v>
+        <v>155</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="I15" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="J15" s="14" t="s">
-        <v>135</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="J15" s="14"/>
       <c r="K15" s="24">
         <v>1</v>
       </c>
       <c r="L15" s="36" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B16) - ROW($B$2)</f>
         <v>14</v>
       </c>
-      <c r="C16" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>135</v>
+      <c r="C16" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="H16" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="I16" s="17" t="s">
+        <v>126</v>
       </c>
       <c r="J16" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K16" s="25">
-        <v>6</v>
-      </c>
-      <c r="L16" s="18"/>
-    </row>
-    <row r="17" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="K16" s="24">
+        <v>1</v>
+      </c>
+      <c r="L16" s="36" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
-        <f>ROW(B17) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C17" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>119</v>
+      <c r="C17" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>116</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J17" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K17" s="22">
-        <v>1</v>
-      </c>
-      <c r="L17" s="37"/>
-    </row>
-    <row r="18" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="K17" s="25">
+        <v>6</v>
+      </c>
+      <c r="L17" s="18"/>
+    </row>
+    <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B18) - ROW($B$2)</f>
         <v>16</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>58</v>
+      <c r="D18" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="G18" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>128</v>
+        <v>79</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>132</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K18" s="23">
-        <v>1</v>
-      </c>
-      <c r="L18" s="18" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="K18" s="22">
+        <v>1</v>
+      </c>
+      <c r="L18" s="37"/>
+    </row>
+    <row r="19" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
-        <f>ROW(B19) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C19" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="E19" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="F19" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="G19" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="H19" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="I19" s="17" t="s">
-        <v>128</v>
+      <c r="C19" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="I19" s="15" t="s">
+        <v>126</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K19" s="24">
-        <v>1</v>
-      </c>
-      <c r="L19" s="37" t="s">
-        <v>155</v>
+        <v>132</v>
+      </c>
+      <c r="K19" s="23">
+        <v>1</v>
+      </c>
+      <c r="L19" s="18" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B20) - ROW($B$2)</f>
         <v>18</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="H20" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="I20" s="15" t="s">
-        <v>128</v>
+      <c r="D20" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="H20" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="I20" s="17" t="s">
+        <v>126</v>
       </c>
       <c r="J20" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K20" s="23">
-        <v>1</v>
-      </c>
-      <c r="L20" s="18" t="s">
-        <v>155</v>
+        <v>132</v>
+      </c>
+      <c r="K20" s="24">
+        <v>2</v>
+      </c>
+      <c r="L20" s="37" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
-        <f>ROW(B21) - ROW($B$2)</f>
         <v>19</v>
       </c>
       <c r="C21" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="J21" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K21" s="22">
-        <v>6</v>
-      </c>
-      <c r="L21" s="37"/>
+      <c r="D21" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>160</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="I21" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="J21" s="14"/>
+      <c r="K21" s="24">
+        <v>1</v>
+      </c>
+      <c r="L21" s="37" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
@@ -1976,31 +1988,31 @@
         <v>12</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J22" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K22" s="23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" s="18" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2009,34 +2021,34 @@
         <f>ROW(B23) - ROW($B$2)</f>
         <v>21</v>
       </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="E23" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="F23" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="G23" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="H23" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="I23" s="17" t="s">
-        <v>128</v>
+      <c r="C23" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>129</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K23" s="24">
-        <v>1</v>
-      </c>
-      <c r="L23" s="37" t="s">
-        <v>155</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="K23" s="22">
+        <v>6</v>
+      </c>
+      <c r="L23" s="37"/>
     </row>
     <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
@@ -2047,453 +2059,533 @@
       <c r="C24" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="G24" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="H24" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="I24" s="10" t="s">
-        <v>132</v>
+      <c r="D24" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="G24" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I24" s="15" t="s">
+        <v>126</v>
       </c>
       <c r="J24" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K24" s="25">
-        <v>1</v>
-      </c>
-      <c r="L24" s="18"/>
-    </row>
-    <row r="25" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="K24" s="23">
+        <v>2</v>
+      </c>
+      <c r="L24" s="18" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
         <v>23</v>
       </c>
-      <c r="C25" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>135</v>
+      <c r="C25" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="H25" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="I25" s="17" t="s">
+        <v>126</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K25" s="22">
-        <v>2</v>
-      </c>
-      <c r="L25" s="37"/>
-    </row>
-    <row r="26" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="K25" s="24">
+        <v>1</v>
+      </c>
+      <c r="L25" s="37" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>137</v>
+        <v>80</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>135</v>
+        <v>108</v>
+      </c>
+      <c r="I26" s="10" t="s">
+        <v>130</v>
       </c>
       <c r="J26" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K26" s="25">
         <v>1</v>
       </c>
       <c r="L26" s="18"/>
     </row>
-    <row r="27" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="12" t="s">
         <v>13</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K27" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L27" s="37"/>
     </row>
-    <row r="28" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="G28" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="I28" s="15" t="s">
-        <v>128</v>
+        <v>13</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>132</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K28" s="23">
-        <v>1</v>
-      </c>
-      <c r="L28" s="18" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="K28" s="25">
+        <v>1</v>
+      </c>
+      <c r="L28" s="18"/>
+    </row>
+    <row r="29" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="12" t="s">
-        <v>14</v>
+      <c r="C29" s="13" t="s">
+        <v>13</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>88</v>
+        <v>65</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>134</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K29" s="22">
         <v>1</v>
       </c>
       <c r="L29" s="37"/>
     </row>
-    <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="G30" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="H30" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="F30" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="G30" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="H30" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="I30" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="I30" s="10" t="s">
-        <v>135</v>
-      </c>
       <c r="J30" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="K30" s="25">
-        <v>1</v>
-      </c>
-      <c r="L30" s="18"/>
-    </row>
-    <row r="31" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="K30" s="23">
+        <v>1</v>
+      </c>
+      <c r="L30" s="18" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="1"/>
       <c r="B31" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>138</v>
+        <v>14</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>140</v>
+        <v>42</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>67</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>135</v>
+        <v>86</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>105</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="I31" s="20" t="s">
-        <v>135</v>
-      </c>
-      <c r="J31" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="K31" s="7">
+        <v>123</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="J31" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="K31" s="22">
         <v>1</v>
       </c>
       <c r="L31" s="37"/>
     </row>
-    <row r="32" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C32" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="F32" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="I32" s="20" t="s">
-        <v>135</v>
-      </c>
-      <c r="J32" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="K32" s="7">
-        <v>1</v>
-      </c>
-      <c r="L32" s="37"/>
-    </row>
-    <row r="33" spans="2:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C32" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="I32" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="J32" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="K32" s="25">
+        <v>1</v>
+      </c>
+      <c r="L32" s="18"/>
+    </row>
+    <row r="33" spans="2:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="11">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C33" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="F33" s="9" t="s">
+      <c r="C33" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="G33" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="I33" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="J33" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="K33" s="9">
-        <v>1</v>
-      </c>
-      <c r="L33" s="18"/>
-    </row>
-    <row r="34" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D33" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="I33" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="J33" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="K33" s="7">
+        <v>1</v>
+      </c>
+      <c r="L33" s="37"/>
+    </row>
+    <row r="34" spans="2:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="11">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C34" s="40" t="s">
-        <v>147</v>
-      </c>
-      <c r="D34" s="43" t="s">
+      <c r="C34" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="E34" s="32" t="s">
-        <v>148</v>
-      </c>
-      <c r="F34" s="33" t="s">
-        <v>135</v>
-      </c>
-      <c r="G34" s="33" t="s">
-        <v>149</v>
-      </c>
-      <c r="H34" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="I34" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="J34" s="29" t="s">
-        <v>141</v>
+      <c r="D34" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="I34" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="J34" s="19" t="s">
+        <v>138</v>
       </c>
       <c r="K34" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L34" s="37"/>
     </row>
-    <row r="35" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="11">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C35" s="41"/>
-      <c r="D35" s="44"/>
-      <c r="E35" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="F35" s="33" t="s">
-        <v>135</v>
-      </c>
-      <c r="G35" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="H35" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="I35" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="J35" s="30" t="s">
+      <c r="C35" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="K35" s="7">
-        <v>2</v>
-      </c>
-      <c r="L35" s="37"/>
+      <c r="D35" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="I35" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="J35" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="K35" s="9">
+        <v>1</v>
+      </c>
+      <c r="L35" s="18"/>
     </row>
     <row r="36" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="11">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C36" s="42"/>
-      <c r="D36" s="45"/>
-      <c r="E36" s="34" t="s">
-        <v>152</v>
-      </c>
-      <c r="F36" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="G36" s="35" t="s">
-        <v>153</v>
-      </c>
-      <c r="H36" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="I36" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="J36" s="31" t="s">
-        <v>141</v>
-      </c>
-      <c r="K36" s="27">
+      <c r="C36" s="40" t="s">
+        <v>144</v>
+      </c>
+      <c r="D36" s="43" t="s">
+        <v>136</v>
+      </c>
+      <c r="E36" s="32" t="s">
+        <v>145</v>
+      </c>
+      <c r="F36" s="33" t="s">
+        <v>132</v>
+      </c>
+      <c r="G36" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="H36" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="I36" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="J36" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="K36" s="7">
+        <v>3</v>
+      </c>
+      <c r="L36" s="37"/>
+    </row>
+    <row r="37" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="11">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="C37" s="41"/>
+      <c r="D37" s="44"/>
+      <c r="E37" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="F37" s="33" t="s">
+        <v>132</v>
+      </c>
+      <c r="G37" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="H37" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="I37" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="J37" s="30" t="s">
+        <v>138</v>
+      </c>
+      <c r="K37" s="7">
+        <v>2</v>
+      </c>
+      <c r="L37" s="37"/>
+    </row>
+    <row r="38" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="11">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="C38" s="42"/>
+      <c r="D38" s="45"/>
+      <c r="E38" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="F38" s="35" t="s">
+        <v>132</v>
+      </c>
+      <c r="G38" s="35" t="s">
+        <v>150</v>
+      </c>
+      <c r="H38" s="35" t="s">
+        <v>132</v>
+      </c>
+      <c r="I38" s="35" t="s">
+        <v>132</v>
+      </c>
+      <c r="J38" s="31" t="s">
+        <v>138</v>
+      </c>
+      <c r="K38" s="27">
         <v>4</v>
       </c>
-      <c r="L36" s="38"/>
+      <c r="L38" s="38"/>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K39">
+        <f>SUM(K3:K38)</f>
+        <v>72</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="I1:L1"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="D36:D38"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="J35" r:id="rId1"/>
-    <hyperlink ref="J36" r:id="rId2"/>
-    <hyperlink ref="J34" r:id="rId3"/>
-    <hyperlink ref="J33" r:id="rId4"/>
-    <hyperlink ref="J32" r:id="rId5"/>
-    <hyperlink ref="J31" r:id="rId6"/>
+    <hyperlink ref="J37" r:id="rId1"/>
+    <hyperlink ref="J38" r:id="rId2"/>
+    <hyperlink ref="J36" r:id="rId3"/>
+    <hyperlink ref="J35" r:id="rId4"/>
+    <hyperlink ref="J34" r:id="rId5"/>
+    <hyperlink ref="J33" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>

</xml_diff>